<commit_message>
calibration example for Jorge
</commit_message>
<xml_diff>
--- a/macros/APSAIA_VIS_2.xlsx
+++ b/macros/APSAIA_VIS_2.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="16">
   <si>
     <t>Run</t>
   </si>
@@ -63,9 +63,6 @@
   <si>
     <t>SiPM289 SiPM290 SiPM377 SiPM378 XARAPUCA</t>
   </si>
-  <si>
-    <t/>
-  </si>
 </sst>
 </file>
 
@@ -74,19 +71,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -122,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -130,7 +121,7 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -141,9 +132,6 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -157,8 +145,8 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -468,24 +456,24 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="11" width="42.29071428571429" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="12" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="13" width="22.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="10" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="42.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="22.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -501,13 +489,13 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -523,7 +511,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -541,23 +529,21 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="6"/>
-      <c r="H2" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="H2" s="1"/>
       <c r="I2" s="6">
         <v>30001</v>
       </c>
-      <c r="J2" s="8">
-        <v>30</v>
-      </c>
-      <c r="K2" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L2" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+      <c r="J2" s="7">
+        <v>30</v>
+      </c>
+      <c r="K2" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L2" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -575,23 +561,21 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="6"/>
-      <c r="H3" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="H3" s="1"/>
       <c r="I3" s="6">
         <v>30001</v>
       </c>
-      <c r="J3" s="8">
-        <v>30</v>
-      </c>
-      <c r="K3" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L3" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+      <c r="J3" s="7">
+        <v>30</v>
+      </c>
+      <c r="K3" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L3" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -608,24 +592,22 @@
         <v>15</v>
       </c>
       <c r="F4" s="1"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="7" t="s">
-        <v>16</v>
-      </c>
+      <c r="G4" s="7"/>
+      <c r="H4" s="1"/>
       <c r="I4" s="6">
         <v>30001</v>
       </c>
-      <c r="J4" s="8">
-        <v>30</v>
-      </c>
-      <c r="K4" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L4" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+      <c r="J4" s="7">
+        <v>30</v>
+      </c>
+      <c r="K4" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L4" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -647,17 +629,17 @@
       <c r="I5" s="6">
         <v>30001</v>
       </c>
-      <c r="J5" s="8">
-        <v>30</v>
-      </c>
-      <c r="K5" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L5" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+      <c r="J5" s="7">
+        <v>30</v>
+      </c>
+      <c r="K5" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L5" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -679,17 +661,17 @@
       <c r="I6" s="6">
         <v>30002</v>
       </c>
-      <c r="J6" s="8">
-        <v>30</v>
-      </c>
-      <c r="K6" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L6" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+      <c r="J6" s="7">
+        <v>30</v>
+      </c>
+      <c r="K6" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L6" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -711,17 +693,17 @@
       <c r="I7" s="6">
         <v>30001</v>
       </c>
-      <c r="J7" s="8">
-        <v>30</v>
-      </c>
-      <c r="K7" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L7" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
+      <c r="J7" s="7">
+        <v>30</v>
+      </c>
+      <c r="K7" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L7" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -738,22 +720,22 @@
         <v>15</v>
       </c>
       <c r="F8" s="1"/>
-      <c r="G8" s="8"/>
+      <c r="G8" s="7"/>
       <c r="H8" s="6"/>
       <c r="I8" s="6">
         <v>30010</v>
       </c>
-      <c r="J8" s="8">
-        <v>30</v>
-      </c>
-      <c r="K8" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L8" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+      <c r="J8" s="7">
+        <v>30</v>
+      </c>
+      <c r="K8" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L8" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -770,22 +752,22 @@
         <v>15</v>
       </c>
       <c r="F9" s="1"/>
-      <c r="G9" s="8"/>
+      <c r="G9" s="7"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6">
         <v>30001</v>
       </c>
-      <c r="J9" s="8">
-        <v>30</v>
-      </c>
-      <c r="K9" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L9" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+      <c r="J9" s="7">
+        <v>30</v>
+      </c>
+      <c r="K9" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L9" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -802,22 +784,22 @@
         <v>15</v>
       </c>
       <c r="F10" s="1"/>
-      <c r="G10" s="8"/>
+      <c r="G10" s="7"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6">
         <v>30001</v>
       </c>
-      <c r="J10" s="8">
-        <v>30</v>
-      </c>
-      <c r="K10" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L10" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+      <c r="J10" s="7">
+        <v>30</v>
+      </c>
+      <c r="K10" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L10" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -839,17 +821,17 @@
       <c r="I11" s="6">
         <v>30001</v>
       </c>
-      <c r="J11" s="8">
-        <v>30</v>
-      </c>
-      <c r="K11" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L11" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+      <c r="J11" s="7">
+        <v>30</v>
+      </c>
+      <c r="K11" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L11" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -871,17 +853,17 @@
       <c r="I12" s="6">
         <v>30001</v>
       </c>
-      <c r="J12" s="8">
-        <v>30</v>
-      </c>
-      <c r="K12" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L12" s="9">
-        <v>25569.0421875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+      <c r="J12" s="7">
+        <v>30</v>
+      </c>
+      <c r="K12" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L12" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -903,14 +885,942 @@
       <c r="I13" s="6">
         <v>30001</v>
       </c>
-      <c r="J13" s="8">
-        <v>30</v>
-      </c>
-      <c r="K13" s="8">
-        <v>1000.02130995131</v>
-      </c>
-      <c r="L13" s="9">
-        <v>25569.0421875</v>
+      <c r="J13" s="7">
+        <v>30</v>
+      </c>
+      <c r="K13" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L13" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+      <c r="A14" s="6">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J14" s="7">
+        <v>30</v>
+      </c>
+      <c r="K14" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L14" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+      <c r="A15" s="6">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J15" s="7">
+        <v>30</v>
+      </c>
+      <c r="K15" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L15" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+      <c r="A16" s="6">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J16" s="7">
+        <v>30</v>
+      </c>
+      <c r="K16" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L16" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+      <c r="A17" s="6">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J17" s="7">
+        <v>30</v>
+      </c>
+      <c r="K17" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L17" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+      <c r="A18" s="6">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J18" s="7">
+        <v>30</v>
+      </c>
+      <c r="K18" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L18" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+      <c r="A19" s="6">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J19" s="7">
+        <v>30</v>
+      </c>
+      <c r="K19" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L19" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+      <c r="A20" s="6">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J20" s="7">
+        <v>30</v>
+      </c>
+      <c r="K20" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L20" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+      <c r="A21" s="6">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J21" s="7">
+        <v>30</v>
+      </c>
+      <c r="K21" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L21" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+      <c r="A22" s="6">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J22" s="7">
+        <v>30</v>
+      </c>
+      <c r="K22" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L22" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+      <c r="A23" s="6">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="1"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J23" s="7">
+        <v>30</v>
+      </c>
+      <c r="K23" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L23" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
+      <c r="A24" s="6">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" s="1"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J24" s="7">
+        <v>30</v>
+      </c>
+      <c r="K24" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L24" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
+      <c r="A25" s="6">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J25" s="7">
+        <v>30</v>
+      </c>
+      <c r="K25" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L25" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
+      <c r="A26" s="6">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="1"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J26" s="7">
+        <v>30</v>
+      </c>
+      <c r="K26" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L26" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
+      <c r="A27" s="6">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="1"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J27" s="7">
+        <v>30</v>
+      </c>
+      <c r="K27" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L27" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
+      <c r="A28" s="6">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" s="1"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J28" s="7">
+        <v>30</v>
+      </c>
+      <c r="K28" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L28" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
+      <c r="A29" s="6">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" s="1"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J29" s="7">
+        <v>30</v>
+      </c>
+      <c r="K29" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L29" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
+      <c r="A30" s="6">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" s="1"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J30" s="7">
+        <v>30</v>
+      </c>
+      <c r="K30" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L30" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
+      <c r="A31" s="6">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="1"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J31" s="7">
+        <v>30</v>
+      </c>
+      <c r="K31" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L31" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25">
+      <c r="A32" s="6">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="1"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J32" s="7">
+        <v>30</v>
+      </c>
+      <c r="K32" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L32" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25">
+      <c r="A33" s="6">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F33" s="1"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J33" s="7">
+        <v>30</v>
+      </c>
+      <c r="K33" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L33" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="17.25">
+      <c r="A34" s="6">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" s="1"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J34" s="7">
+        <v>30</v>
+      </c>
+      <c r="K34" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L34" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="17.25">
+      <c r="A35" s="6">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F35" s="1"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J35" s="7">
+        <v>30</v>
+      </c>
+      <c r="K35" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L35" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="17.25">
+      <c r="A36" s="6">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J36" s="7">
+        <v>30</v>
+      </c>
+      <c r="K36" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L36" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="17.25">
+      <c r="A37" s="6">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J37" s="7">
+        <v>30</v>
+      </c>
+      <c r="K37" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L37" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="17.25">
+      <c r="A38" s="6">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" s="1"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J38" s="7">
+        <v>30</v>
+      </c>
+      <c r="K38" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L38" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="17.25">
+      <c r="A39" s="6">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F39" s="1"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J39" s="7">
+        <v>30</v>
+      </c>
+      <c r="K39" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L39" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="17.25">
+      <c r="A40" s="6">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" s="1"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J40" s="7">
+        <v>30</v>
+      </c>
+      <c r="K40" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L40" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="17.25">
+      <c r="A41" s="6">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="1"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J41" s="7">
+        <v>30</v>
+      </c>
+      <c r="K41" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L41" s="8">
+        <v>25569.041962604166</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="17.25">
+      <c r="A42" s="6">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F42" s="1"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6">
+        <v>30001</v>
+      </c>
+      <c r="J42" s="7">
+        <v>30</v>
+      </c>
+      <c r="K42" s="7">
+        <v>1000.02130995131</v>
+      </c>
+      <c r="L42" s="8">
+        <v>25569.041962604166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>